<commit_message>
Removing unwanted New technology
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_NewTechs.xlsx
+++ b/SubRES_TMPL/SubRES_NewTechs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98AFC909-2EA9-4EDC-9E2A-898492BADD7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC9944C-77B9-4EFA-9682-1653773D6577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ELC" sheetId="4" r:id="rId1"/>
@@ -41,22 +41,13 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={7B12096A-3111-40C7-94B2-C82D924DD46E}</author>
     <author>tc={9A97F4CE-0467-4677-8B57-18CDF16525F8}</author>
     <author>tc={D5D738E1-1D01-4540-9F11-10D499C0D688}</author>
     <author>tc={A3E54751-892C-48B6-A7DF-516DEC7FED8F}</author>
     <author>tc={7634B8F0-2D0A-458A-9170-2B40B7F18B83}</author>
   </authors>
   <commentList>
-    <comment ref="O14" authorId="0" shapeId="0" xr:uid="{7B12096A-3111-40C7-94B2-C82D924DD46E}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Fermil pole väärtust andnud</t>
-      </text>
-    </comment>
-    <comment ref="G15" authorId="1" shapeId="0" xr:uid="{9A97F4CE-0467-4677-8B57-18CDF16525F8}">
+    <comment ref="G14" authorId="0" shapeId="0" xr:uid="{9A97F4CE-0467-4677-8B57-18CDF16525F8}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -64,7 +55,7 @@
     Google otsing</t>
       </text>
     </comment>
-    <comment ref="I15" authorId="2" shapeId="0" xr:uid="{D5D738E1-1D01-4540-9F11-10D499C0D688}">
+    <comment ref="I14" authorId="1" shapeId="0" xr:uid="{D5D738E1-1D01-4540-9F11-10D499C0D688}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -72,7 +63,7 @@
     18 MUSD/MW</t>
       </text>
     </comment>
-    <comment ref="J15" authorId="3" shapeId="0" xr:uid="{A3E54751-892C-48B6-A7DF-516DEC7FED8F}">
+    <comment ref="J14" authorId="2" shapeId="0" xr:uid="{A3E54751-892C-48B6-A7DF-516DEC7FED8F}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -80,7 +71,7 @@
     Fermil oli antud 27 €/MWh kohta, mis sisaldas 6 €/Mwh kütusekulu </t>
       </text>
     </comment>
-    <comment ref="K15" authorId="4" shapeId="0" xr:uid="{7634B8F0-2D0A-458A-9170-2B40B7F18B83}">
+    <comment ref="K14" authorId="3" shapeId="0" xr:uid="{7634B8F0-2D0A-458A-9170-2B40B7F18B83}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -93,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="109">
   <si>
     <t>~FI_T</t>
   </si>
@@ -335,9 +326,6 @@
     <t>ELE</t>
   </si>
   <si>
-    <t>ELCCOA</t>
-  </si>
-  <si>
     <t>ELCGAS</t>
   </si>
   <si>
@@ -348,12 +336,6 @@
   </si>
   <si>
     <t>Yes</t>
-  </si>
-  <si>
-    <t>Power Plants New 1 - Solid Fuels</t>
-  </si>
-  <si>
-    <t>ELCTNCOA01</t>
   </si>
   <si>
     <t>ELCSOL</t>
@@ -438,10 +420,10 @@
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="\Te\x\t"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="\Te\x\t"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -583,19 +565,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <charset val="186"/>
     </font>
     <font>
       <sz val="10"/>
@@ -850,25 +819,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="20" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="20" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="20" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="20" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="32" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="15" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="32" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="15" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="15" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -1372,19 +1341,16 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="O14" dT="2026-10-19T11:06:02.02" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{7B12096A-3111-40C7-94B2-C82D924DD46E}">
-    <text>Fermil pole väärtust andnud</text>
-  </threadedComment>
-  <threadedComment ref="G15" dT="2026-10-19T10:21:04.55" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{9A97F4CE-0467-4677-8B57-18CDF16525F8}">
+  <threadedComment ref="G14" dT="2026-10-19T10:21:04.55" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{9A97F4CE-0467-4677-8B57-18CDF16525F8}">
     <text>Google otsing</text>
   </threadedComment>
-  <threadedComment ref="I15" dT="2026-10-19T10:23:13.18" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{D5D738E1-1D01-4540-9F11-10D499C0D688}">
+  <threadedComment ref="I14" dT="2026-10-19T10:23:13.18" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{D5D738E1-1D01-4540-9F11-10D499C0D688}">
     <text>18 MUSD/MW</text>
   </threadedComment>
-  <threadedComment ref="J15" dT="2026-10-19T10:37:46.35" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{A3E54751-892C-48B6-A7DF-516DEC7FED8F}">
+  <threadedComment ref="J14" dT="2026-10-19T10:37:46.35" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{A3E54751-892C-48B6-A7DF-516DEC7FED8F}">
     <text xml:space="preserve">Fermil oli antud 27 €/MWh kohta, mis sisaldas 6 €/Mwh kütusekulu </text>
   </threadedComment>
-  <threadedComment ref="K15" dT="2026-10-19T10:40:37.40" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{7634B8F0-2D0A-458A-9170-2B40B7F18B83}">
+  <threadedComment ref="K14" dT="2026-10-19T10:40:37.40" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{7634B8F0-2D0A-458A-9170-2B40B7F18B83}">
     <text>google</text>
   </threadedComment>
 </ThreadedComments>
@@ -1393,7 +1359,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:Y32"/>
+  <dimension ref="A1:Y31"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" style="20" customWidth="1"/>
@@ -1469,7 +1435,7 @@
         <v>50</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>52</v>
@@ -1616,7 +1582,7 @@
         <v>4</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F11" s="14" t="s">
         <v>15</v>
@@ -1640,13 +1606,13 @@
         <v>66</v>
       </c>
       <c r="M11" s="13" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="N11" s="13" t="s">
         <v>67</v>
       </c>
       <c r="O11" s="13" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="P11" s="21"/>
       <c r="Q11" s="30" t="s">
@@ -1689,7 +1655,7 @@
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="15" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>37</v>
@@ -1707,7 +1673,7 @@
         <v>41</v>
       </c>
       <c r="L12" s="15" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="M12" s="15" t="s">
         <v>38</v>
@@ -1716,7 +1682,7 @@
         <v>71</v>
       </c>
       <c r="O12" s="39" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="Q12" s="33" t="s">
         <v>72</v>
@@ -1763,7 +1729,7 @@
         <v>76</v>
       </c>
       <c r="K13" s="17" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L13" s="17" t="s">
         <v>77</v>
@@ -1774,7 +1740,7 @@
       <c r="N13" s="17"/>
       <c r="O13" s="17"/>
       <c r="Q13" s="32" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R13" s="32"/>
       <c r="S13" s="32"/>
@@ -1786,33 +1752,40 @@
       <c r="Y13" s="32"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="B14" s="20" t="str">
-        <f>S14</f>
-        <v>ELCTNCOA01</v>
+      <c r="B14" s="36" t="str">
+        <f>$S$14</f>
+        <v>ELC_FERMI_SMR</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="D14" s="20" t="s">
         <v>47</v>
       </c>
+      <c r="E14" s="20">
+        <v>2036</v>
+      </c>
+      <c r="F14" s="20">
+        <v>2036</v>
+      </c>
       <c r="G14" s="22">
-        <v>0.42</v>
-      </c>
-      <c r="H14" s="22">
-        <v>0.85</v>
+        <v>0.3</v>
+      </c>
+      <c r="H14" s="20">
+        <v>0.92</v>
       </c>
       <c r="I14" s="20">
-        <v>1650</v>
+        <v>15000</v>
       </c>
       <c r="J14" s="22">
-        <v>35</v>
+        <f>21*H14*8760*1000/1000000</f>
+        <v>169.2432</v>
       </c>
       <c r="K14" s="22">
-        <v>0.4</v>
+        <v>3.15</v>
       </c>
       <c r="L14" s="20">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="M14" s="20">
         <v>31.536000000000001</v>
@@ -1821,48 +1794,45 @@
         <v>1</v>
       </c>
       <c r="O14" s="22"/>
-      <c r="Q14" s="34" t="s">
+      <c r="Q14" s="35" t="s">
         <v>79</v>
       </c>
       <c r="R14" s="34"/>
-      <c r="S14" s="34" t="s">
-        <v>86</v>
+      <c r="S14" s="36" t="s">
+        <v>92</v>
       </c>
       <c r="T14" s="34" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="U14" s="34" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="V14" s="34" t="s">
         <v>51</v>
       </c>
       <c r="W14" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="X14" s="34"/>
       <c r="Y14" s="34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="B15" s="36" t="str">
-        <f>$S$15</f>
+        <f>$S$14</f>
         <v>ELC_FERMI_SMR</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D15" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E15" s="20">
-        <v>2036</v>
-      </c>
-      <c r="F15" s="20">
-        <v>2036</v>
-      </c>
-      <c r="G15" s="22">
+        <v>2040</v>
+      </c>
+      <c r="G15" s="20">
         <v>0.3</v>
       </c>
       <c r="H15" s="20">
@@ -1872,8 +1842,8 @@
         <v>15000</v>
       </c>
       <c r="J15" s="22">
-        <f>21*H15*8760*1000/1000000</f>
-        <v>169.2432</v>
+        <f t="shared" ref="J15:J16" si="0">169243*1000/1000000</f>
+        <v>169.24299999999999</v>
       </c>
       <c r="K15" s="22">
         <v>3.15</v>
@@ -1888,43 +1858,42 @@
         <v>1</v>
       </c>
       <c r="O15" s="22"/>
-      <c r="Q15" s="35" t="s">
+      <c r="Q15" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="R15" s="34"/>
-      <c r="S15" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="T15" s="34" t="s">
+      <c r="S15" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="T15" t="s">
         <v>94</v>
       </c>
       <c r="U15" s="34" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="V15" s="34" t="s">
         <v>51</v>
       </c>
       <c r="W15" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="X15" s="34"/>
       <c r="Y15" s="34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.2">
       <c r="B16" s="36" t="str">
-        <f>$S$15</f>
+        <f>$S$14</f>
         <v>ELC_FERMI_SMR</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D16" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E16" s="20">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="G16" s="20">
         <v>0.3</v>
@@ -1936,7 +1905,7 @@
         <v>15000</v>
       </c>
       <c r="J16" s="22">
-        <f t="shared" ref="J16:J17" si="0">169243*1000/1000000</f>
+        <f t="shared" si="0"/>
         <v>169.24299999999999</v>
       </c>
       <c r="K16" s="22">
@@ -1955,58 +1924,62 @@
       <c r="Q16" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="S16" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="T16" t="s">
-        <v>97</v>
+      <c r="S16" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="T16" s="38" t="s">
+        <v>107</v>
       </c>
       <c r="U16" s="34" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="V16" s="34" t="s">
         <v>51</v>
       </c>
       <c r="W16" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="X16" s="34"/>
       <c r="Y16" s="34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B17" s="36" t="str">
+      <c r="B17" s="20" t="str">
         <f>$S$15</f>
-        <v>ELC_FERMI_SMR</v>
+        <v>ELC_CCGT_PP</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D17" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E17" s="20">
-        <v>2050</v>
+        <v>2030</v>
+      </c>
+      <c r="F17" s="20">
+        <v>2030</v>
       </c>
       <c r="G17" s="20">
-        <v>0.3</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="H17" s="20">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="I17" s="20">
-        <v>15000</v>
+        <f>1.2*1000</f>
+        <v>1200</v>
       </c>
       <c r="J17" s="22">
-        <f t="shared" si="0"/>
-        <v>169.24299999999999</v>
-      </c>
-      <c r="K17" s="22">
-        <v>3.15</v>
+        <f>39143*1000/1000000</f>
+        <v>39.143000000000001</v>
+      </c>
+      <c r="K17" s="20">
+        <v>5.9</v>
       </c>
       <c r="L17" s="20">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="M17" s="20">
         <v>31.536000000000001</v>
@@ -2014,46 +1987,45 @@
       <c r="N17" s="22">
         <v>1</v>
       </c>
-      <c r="O17" s="22"/>
+      <c r="O17" s="22">
+        <v>2.5</v>
+      </c>
       <c r="Q17" s="38" t="s">
         <v>79</v>
       </c>
       <c r="S17" s="38" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="T17" s="38" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="U17" s="34" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="V17" s="34" t="s">
         <v>51</v>
       </c>
       <c r="W17" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="X17" s="34"/>
       <c r="Y17" s="34" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="18" spans="2:25" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="2:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="20" t="str">
-        <f>$S$16</f>
+        <f>$S$15</f>
         <v>ELC_CCGT_PP</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D18" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E18" s="20">
-        <v>2030</v>
-      </c>
-      <c r="F18" s="20">
-        <v>2030</v>
+        <v>2040</v>
       </c>
       <c r="G18" s="20">
         <v>0.56000000000000005</v>
@@ -2066,7 +2038,7 @@
         <v>1200</v>
       </c>
       <c r="J18" s="22">
-        <f>39143*1000/1000000</f>
+        <f t="shared" ref="J18:J19" si="1">39143*1000/1000000</f>
         <v>39.143000000000001</v>
       </c>
       <c r="K18" s="20">
@@ -2087,39 +2059,39 @@
       <c r="Q18" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="S18" s="38" t="s">
+      <c r="S18" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="T18" s="38" t="s">
-        <v>101</v>
+      <c r="T18" s="20" t="s">
+        <v>103</v>
       </c>
       <c r="U18" s="34" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="V18" s="34" t="s">
         <v>51</v>
       </c>
       <c r="W18" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="X18" s="34"/>
       <c r="Y18" s="34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="2:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="20" t="str">
-        <f>$S$16</f>
+        <f>$S$15</f>
         <v>ELC_CCGT_PP</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D19" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E19" s="20">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="G19" s="20">
         <v>0.56000000000000005</v>
@@ -2132,7 +2104,7 @@
         <v>1200</v>
       </c>
       <c r="J19" s="22">
-        <f t="shared" ref="J19:J20" si="1">39143*1000/1000000</f>
+        <f t="shared" si="1"/>
         <v>39.143000000000001</v>
       </c>
       <c r="K19" s="20">
@@ -2153,56 +2125,59 @@
       <c r="Q19" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="S19" s="20" t="s">
+      <c r="S19" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="T19" s="20" t="s">
+      <c r="T19" s="38" t="s">
         <v>106</v>
       </c>
       <c r="U19" s="34" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="V19" s="34" t="s">
         <v>51</v>
       </c>
       <c r="W19" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="X19" s="34"/>
       <c r="Y19" s="34" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="20" spans="2:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B20" s="20" t="str">
         <f>$S$16</f>
-        <v>ELC_CCGT_PP</v>
+        <v>ELC_OCGT_PP</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D20" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E20" s="20">
-        <v>2050</v>
+        <v>2030</v>
+      </c>
+      <c r="F20" s="20">
+        <v>2030</v>
       </c>
       <c r="G20" s="20">
-        <v>0.56000000000000005</v>
+        <v>0.4</v>
       </c>
       <c r="H20" s="20">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="I20" s="20">
-        <f>1.2*1000</f>
-        <v>1200</v>
+        <f>0.6*1000</f>
+        <v>600</v>
       </c>
       <c r="J20" s="22">
-        <f t="shared" si="1"/>
-        <v>39.143000000000001</v>
-      </c>
-      <c r="K20" s="20">
-        <v>5.9</v>
+        <f>10778*1000/1000000</f>
+        <v>10.778</v>
+      </c>
+      <c r="K20" s="37">
+        <v>6</v>
       </c>
       <c r="L20" s="20">
         <v>25</v>
@@ -2213,48 +2188,23 @@
       <c r="N20" s="22">
         <v>1</v>
       </c>
-      <c r="O20" s="22">
-        <v>2.5</v>
-      </c>
-      <c r="Q20" s="38" t="s">
-        <v>79</v>
-      </c>
-      <c r="S20" s="38" t="s">
-        <v>108</v>
-      </c>
-      <c r="T20" s="38" t="s">
-        <v>109</v>
-      </c>
-      <c r="U20" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="V20" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="W20" t="s">
-        <v>93</v>
-      </c>
-      <c r="X20" s="34"/>
-      <c r="Y20" s="34" t="s">
-        <v>84</v>
+      <c r="O20" s="20">
+        <v>0.2</v>
       </c>
     </row>
     <row r="21" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B21" s="20" t="str">
-        <f>$S$17</f>
+        <f t="shared" ref="B21:B22" si="2">$S$16</f>
         <v>ELC_OCGT_PP</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D21" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E21" s="20">
-        <v>2030</v>
-      </c>
-      <c r="F21" s="20">
-        <v>2030</v>
+        <v>2040</v>
       </c>
       <c r="G21" s="20">
         <v>0.4</v>
@@ -2263,11 +2213,11 @@
         <v>0.99</v>
       </c>
       <c r="I21" s="20">
-        <f>0.6*1000</f>
+        <f t="shared" ref="I21:I22" si="3">0.6*1000</f>
         <v>600</v>
       </c>
       <c r="J21" s="22">
-        <f>10778*1000/1000000</f>
+        <f t="shared" ref="J21:J22" si="4">10778*1000/1000000</f>
         <v>10.778</v>
       </c>
       <c r="K21" s="37">
@@ -2288,17 +2238,17 @@
     </row>
     <row r="22" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="str">
-        <f t="shared" ref="B22:B23" si="2">$S$17</f>
+        <f t="shared" si="2"/>
         <v>ELC_OCGT_PP</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D22" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E22" s="20">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="G22" s="20">
         <v>0.4</v>
@@ -2307,11 +2257,11 @@
         <v>0.99</v>
       </c>
       <c r="I22" s="20">
-        <f t="shared" ref="I22:I23" si="3">0.6*1000</f>
+        <f t="shared" si="3"/>
         <v>600</v>
       </c>
       <c r="J22" s="22">
-        <f t="shared" ref="J22:J23" si="4">10778*1000/1000000</f>
+        <f t="shared" si="4"/>
         <v>10.778</v>
       </c>
       <c r="K22" s="37">
@@ -2332,37 +2282,40 @@
     </row>
     <row r="23" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B23" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v>ELC_OCGT_PP</v>
+        <f>$S$17</f>
+        <v>ELC_PV_UTIL</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D23" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E23" s="20">
-        <v>2050</v>
+        <v>2030</v>
+      </c>
+      <c r="F23" s="20">
+        <v>2030</v>
       </c>
       <c r="G23" s="20">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H23" s="20">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="I23" s="20">
-        <f t="shared" si="3"/>
-        <v>600</v>
+        <f>0.7*1000</f>
+        <v>700</v>
       </c>
       <c r="J23" s="22">
-        <f t="shared" si="4"/>
-        <v>10.778</v>
-      </c>
-      <c r="K23" s="37">
-        <v>6</v>
+        <f>12601*1000/1000000</f>
+        <v>12.601000000000001</v>
+      </c>
+      <c r="K23" s="20">
+        <v>0</v>
       </c>
       <c r="L23" s="20">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="M23" s="20">
         <v>31.536000000000001</v>
@@ -2371,25 +2324,22 @@
         <v>1</v>
       </c>
       <c r="O23" s="20">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B24" s="20" t="str">
-        <f>$S$18</f>
+        <f t="shared" ref="B24:B25" si="5">$S$17</f>
         <v>ELC_PV_UTIL</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D24" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="20">
-        <v>2030</v>
-      </c>
-      <c r="F24" s="20">
-        <v>2030</v>
+        <v>2040</v>
       </c>
       <c r="G24" s="20">
         <v>1</v>
@@ -2398,11 +2348,11 @@
         <v>1</v>
       </c>
       <c r="I24" s="20">
-        <f>0.7*1000</f>
+        <f t="shared" ref="I24:I25" si="6">0.7*1000</f>
         <v>700</v>
       </c>
       <c r="J24" s="22">
-        <f>12601*1000/1000000</f>
+        <f t="shared" ref="J24:J25" si="7">12601*1000/1000000</f>
         <v>12.601000000000001</v>
       </c>
       <c r="K24" s="20">
@@ -2423,17 +2373,17 @@
     </row>
     <row r="25" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B25" s="20" t="str">
-        <f t="shared" ref="B25:B26" si="5">$S$18</f>
+        <f t="shared" si="5"/>
         <v>ELC_PV_UTIL</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D25" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E25" s="20">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="G25" s="20">
         <v>1</v>
@@ -2442,11 +2392,11 @@
         <v>1</v>
       </c>
       <c r="I25" s="20">
-        <f t="shared" ref="I25:I26" si="6">0.7*1000</f>
+        <f t="shared" si="6"/>
         <v>700</v>
       </c>
       <c r="J25" s="22">
-        <f t="shared" ref="J25:J26" si="7">12601*1000/1000000</f>
+        <f t="shared" si="7"/>
         <v>12.601000000000001</v>
       </c>
       <c r="K25" s="20">
@@ -2467,37 +2417,40 @@
     </row>
     <row r="26" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="str">
-        <f t="shared" si="5"/>
-        <v>ELC_PV_UTIL</v>
+        <f>$S$18</f>
+        <v>ELC_WON_PP</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D26" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E26" s="20">
-        <v>2050</v>
+        <v>2030</v>
+      </c>
+      <c r="F26" s="20">
+        <v>2030</v>
       </c>
       <c r="G26" s="20">
         <v>1</v>
       </c>
       <c r="H26" s="20">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="I26" s="20">
-        <f t="shared" si="6"/>
-        <v>700</v>
+        <f>1.5*1000</f>
+        <v>1500</v>
       </c>
       <c r="J26" s="22">
-        <f t="shared" si="7"/>
-        <v>12.601000000000001</v>
+        <f>21843*1000/1000000</f>
+        <v>21.843</v>
       </c>
       <c r="K26" s="20">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="L26" s="20">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="M26" s="20">
         <v>31.536000000000001</v>
@@ -2506,25 +2459,22 @@
         <v>1</v>
       </c>
       <c r="O26" s="20">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="27" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B27" s="20" t="str">
-        <f>$S$19</f>
+        <f t="shared" ref="B27:B28" si="8">$S$18</f>
         <v>ELC_WON_PP</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D27" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E27" s="20">
-        <v>2030</v>
-      </c>
-      <c r="F27" s="20">
-        <v>2030</v>
+        <v>2040</v>
       </c>
       <c r="G27" s="20">
         <v>1</v>
@@ -2533,11 +2483,11 @@
         <v>0.97</v>
       </c>
       <c r="I27" s="20">
-        <f>1.5*1000</f>
+        <f t="shared" ref="I27:I28" si="9">1.5*1000</f>
         <v>1500</v>
       </c>
       <c r="J27" s="22">
-        <f>21843*1000/1000000</f>
+        <f t="shared" ref="J27:J28" si="10">21843*1000/1000000</f>
         <v>21.843</v>
       </c>
       <c r="K27" s="20">
@@ -2558,17 +2508,17 @@
     </row>
     <row r="28" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="str">
-        <f t="shared" ref="B28:B29" si="8">$S$19</f>
+        <f t="shared" si="8"/>
         <v>ELC_WON_PP</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D28" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E28" s="20">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="G28" s="20">
         <v>1</v>
@@ -2577,11 +2527,11 @@
         <v>0.97</v>
       </c>
       <c r="I28" s="20">
-        <f t="shared" ref="I28:I29" si="9">1.5*1000</f>
+        <f t="shared" si="9"/>
         <v>1500</v>
       </c>
       <c r="J28" s="22">
-        <f t="shared" ref="J28:J29" si="10">21843*1000/1000000</f>
+        <f t="shared" si="10"/>
         <v>21.843</v>
       </c>
       <c r="K28" s="20">
@@ -2602,37 +2552,40 @@
     </row>
     <row r="29" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B29" s="20" t="str">
-        <f t="shared" si="8"/>
-        <v>ELC_WON_PP</v>
+        <f>$S$19</f>
+        <v>ELC_WOF_PP</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D29" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E29" s="20">
-        <v>2050</v>
+        <v>2030</v>
+      </c>
+      <c r="F29" s="20">
+        <v>2030</v>
       </c>
       <c r="G29" s="20">
         <v>1</v>
       </c>
       <c r="H29" s="20">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="I29" s="20">
-        <f t="shared" si="9"/>
-        <v>1500</v>
+        <f>3.5*1000</f>
+        <v>3500</v>
       </c>
       <c r="J29" s="22">
-        <f t="shared" si="10"/>
-        <v>21.843</v>
+        <f>55278*1000/1000000</f>
+        <v>55.277999999999999</v>
       </c>
       <c r="K29" s="20">
-        <v>2.6</v>
+        <v>5.5</v>
       </c>
       <c r="L29" s="20">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M29" s="20">
         <v>31.536000000000001</v>
@@ -2641,25 +2594,22 @@
         <v>1</v>
       </c>
       <c r="O29" s="20">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="30" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="str">
-        <f>$S$20</f>
+        <f>$S$19</f>
         <v>ELC_WOF_PP</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D30" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E30" s="20">
-        <v>2030</v>
-      </c>
-      <c r="F30" s="20">
-        <v>2030</v>
+        <v>2040</v>
       </c>
       <c r="G30" s="20">
         <v>1</v>
@@ -2668,11 +2618,11 @@
         <v>0.98</v>
       </c>
       <c r="I30" s="20">
-        <f>3.5*1000</f>
+        <f t="shared" ref="I30:I31" si="11">3.5*1000</f>
         <v>3500</v>
       </c>
       <c r="J30" s="22">
-        <f>55278*1000/1000000</f>
+        <f t="shared" ref="J30:J31" si="12">55278*1000/1000000</f>
         <v>55.277999999999999</v>
       </c>
       <c r="K30" s="20">
@@ -2693,17 +2643,17 @@
     </row>
     <row r="31" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B31" s="20" t="str">
-        <f>$S$20</f>
+        <f>$S$19</f>
         <v>ELC_WOF_PP</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D31" s="20" t="s">
         <v>47</v>
       </c>
       <c r="E31" s="20">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="G31" s="20">
         <v>1</v>
@@ -2712,11 +2662,11 @@
         <v>0.98</v>
       </c>
       <c r="I31" s="20">
-        <f t="shared" ref="I31:I32" si="11">3.5*1000</f>
+        <f t="shared" si="11"/>
         <v>3500</v>
       </c>
       <c r="J31" s="22">
-        <f t="shared" ref="J31:J32" si="12">55278*1000/1000000</f>
+        <f t="shared" si="12"/>
         <v>55.277999999999999</v>
       </c>
       <c r="K31" s="20">
@@ -2732,50 +2682,6 @@
         <v>1</v>
       </c>
       <c r="O31" s="20">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="32" spans="2:25" x14ac:dyDescent="0.2">
-      <c r="B32" s="20" t="str">
-        <f>$S$20</f>
-        <v>ELC_WOF_PP</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="D32" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="E32" s="20">
-        <v>2050</v>
-      </c>
-      <c r="G32" s="20">
-        <v>1</v>
-      </c>
-      <c r="H32" s="20">
-        <v>0.98</v>
-      </c>
-      <c r="I32" s="20">
-        <f t="shared" si="11"/>
-        <v>3500</v>
-      </c>
-      <c r="J32" s="22">
-        <f t="shared" si="12"/>
-        <v>55.277999999999999</v>
-      </c>
-      <c r="K32" s="20">
-        <v>5.5</v>
-      </c>
-      <c r="L32" s="20">
-        <v>30</v>
-      </c>
-      <c r="M32" s="20">
-        <v>31.536000000000001</v>
-      </c>
-      <c r="N32" s="22">
-        <v>1</v>
-      </c>
-      <c r="O32" s="20">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
FIxing utilisation factor of new wind and solar plants
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_NewTechs.xlsx
+++ b/SubRES_TMPL/SubRES_NewTechs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC9944C-77B9-4EFA-9682-1653773D6577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{309F4561-CB01-4649-B761-C06A2C8B23CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ELC" sheetId="4" r:id="rId1"/>
@@ -1401,7 +1401,7 @@
       <c r="X2" s="27"/>
       <c r="Y2" s="27"/>
     </row>
-    <row r="3" spans="1:25" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="B3" s="19" t="s">
         <v>42</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>1</v>
       </c>
       <c r="H23" s="20">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I23" s="20">
         <f>0.7*1000</f>
@@ -2321,7 +2321,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="N23" s="22">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="O23" s="20">
         <v>0.5</v>
@@ -2345,7 +2345,7 @@
         <v>1</v>
       </c>
       <c r="H24" s="20">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I24" s="20">
         <f t="shared" ref="I24:I25" si="6">0.7*1000</f>
@@ -2365,7 +2365,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="N24" s="22">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="O24" s="20">
         <v>0.5</v>
@@ -2389,7 +2389,7 @@
         <v>1</v>
       </c>
       <c r="H25" s="20">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I25" s="20">
         <f t="shared" si="6"/>
@@ -2409,7 +2409,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="N25" s="22">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="O25" s="20">
         <v>0.5</v>
@@ -2436,7 +2436,7 @@
         <v>1</v>
       </c>
       <c r="H26" s="20">
-        <v>0.97</v>
+        <v>0.3</v>
       </c>
       <c r="I26" s="20">
         <f>1.5*1000</f>
@@ -2456,7 +2456,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="N26" s="22">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="O26" s="20">
         <v>1.5</v>
@@ -2480,7 +2480,7 @@
         <v>1</v>
       </c>
       <c r="H27" s="20">
-        <v>0.97</v>
+        <v>0.3</v>
       </c>
       <c r="I27" s="20">
         <f t="shared" ref="I27:I28" si="9">1.5*1000</f>
@@ -2500,7 +2500,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="N27" s="22">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="O27" s="20">
         <v>1.5</v>
@@ -2524,7 +2524,7 @@
         <v>1</v>
       </c>
       <c r="H28" s="20">
-        <v>0.97</v>
+        <v>0.3</v>
       </c>
       <c r="I28" s="20">
         <f t="shared" si="9"/>
@@ -2544,7 +2544,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="N28" s="22">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="O28" s="20">
         <v>1.5</v>
@@ -2571,7 +2571,7 @@
         <v>1</v>
       </c>
       <c r="H29" s="20">
-        <v>0.98</v>
+        <v>0.3</v>
       </c>
       <c r="I29" s="20">
         <f>3.5*1000</f>
@@ -2591,7 +2591,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="N29" s="22">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="O29" s="20">
         <v>3.5</v>
@@ -2615,7 +2615,7 @@
         <v>1</v>
       </c>
       <c r="H30" s="20">
-        <v>0.98</v>
+        <v>0.3</v>
       </c>
       <c r="I30" s="20">
         <f t="shared" ref="I30:I31" si="11">3.5*1000</f>
@@ -2635,7 +2635,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="N30" s="22">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="O30" s="20">
         <v>3.5</v>
@@ -2659,7 +2659,7 @@
         <v>1</v>
       </c>
       <c r="H31" s="20">
-        <v>0.98</v>
+        <v>0.3</v>
       </c>
       <c r="I31" s="20">
         <f t="shared" si="11"/>
@@ -2679,7 +2679,7 @@
         <v>31.536000000000001</v>
       </c>
       <c r="N31" s="22">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="O31" s="20">
         <v>3.5</v>

</xml_diff>

<commit_message>
FIxing cap2act for new technologies
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_NewTechs.xlsx
+++ b/SubRES_TMPL/SubRES_NewTechs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{309F4561-CB01-4649-B761-C06A2C8B23CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66004E25-ED8F-4478-B1BA-EF53FDD0DE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1401,7 +1401,7 @@
       <c r="X2" s="27"/>
       <c r="Y2" s="27"/>
     </row>
-    <row r="3" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15" x14ac:dyDescent="0.25">
       <c r="B3" s="19" t="s">
         <v>42</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>60</v>
       </c>
       <c r="M14" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N14" s="22">
         <v>1</v>
@@ -1852,7 +1852,7 @@
         <v>60</v>
       </c>
       <c r="M15" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N15" s="22">
         <v>1</v>
@@ -1915,7 +1915,7 @@
         <v>60</v>
       </c>
       <c r="M16" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N16" s="22">
         <v>1</v>
@@ -1982,7 +1982,7 @@
         <v>25</v>
       </c>
       <c r="M17" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N17" s="22">
         <v>1</v>
@@ -2048,7 +2048,7 @@
         <v>25</v>
       </c>
       <c r="M18" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N18" s="22">
         <v>1</v>
@@ -2114,7 +2114,7 @@
         <v>25</v>
       </c>
       <c r="M19" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N19" s="22">
         <v>1</v>
@@ -2183,7 +2183,7 @@
         <v>25</v>
       </c>
       <c r="M20" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N20" s="22">
         <v>1</v>
@@ -2227,7 +2227,7 @@
         <v>25</v>
       </c>
       <c r="M21" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N21" s="22">
         <v>1</v>
@@ -2271,7 +2271,7 @@
         <v>25</v>
       </c>
       <c r="M22" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N22" s="22">
         <v>1</v>
@@ -2318,7 +2318,7 @@
         <v>40</v>
       </c>
       <c r="M23" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N23" s="22">
         <v>0.15</v>
@@ -2362,7 +2362,7 @@
         <v>40</v>
       </c>
       <c r="M24" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N24" s="22">
         <v>0.15</v>
@@ -2406,7 +2406,7 @@
         <v>40</v>
       </c>
       <c r="M25" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N25" s="22">
         <v>0.15</v>
@@ -2453,7 +2453,7 @@
         <v>27</v>
       </c>
       <c r="M26" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N26" s="22">
         <v>0.4</v>
@@ -2497,7 +2497,7 @@
         <v>27</v>
       </c>
       <c r="M27" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N27" s="22">
         <v>0.4</v>
@@ -2541,7 +2541,7 @@
         <v>27</v>
       </c>
       <c r="M28" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N28" s="22">
         <v>0.4</v>
@@ -2588,7 +2588,7 @@
         <v>30</v>
       </c>
       <c r="M29" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N29" s="22">
         <v>0.4</v>
@@ -2632,7 +2632,7 @@
         <v>30</v>
       </c>
       <c r="M30" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N30" s="22">
         <v>0.4</v>
@@ -2676,7 +2676,7 @@
         <v>30</v>
       </c>
       <c r="M31" s="20">
-        <v>31.536000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="N31" s="22">
         <v>0.4</v>

</xml_diff>

<commit_message>
Changing start year of new technologies
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_NewTechs.xlsx
+++ b/SubRES_TMPL/SubRES_NewTechs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66004E25-ED8F-4478-B1BA-EF53FDD0DE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED673232-5F8D-4EB7-8769-7EC4F8A479E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ELC" sheetId="4" r:id="rId1"/>
@@ -1959,7 +1959,7 @@
         <v>2030</v>
       </c>
       <c r="F17" s="20">
-        <v>2030</v>
+        <v>2027</v>
       </c>
       <c r="G17" s="20">
         <v>0.56000000000000005</v>
@@ -2160,7 +2160,7 @@
         <v>2030</v>
       </c>
       <c r="F20" s="20">
-        <v>2030</v>
+        <v>2027</v>
       </c>
       <c r="G20" s="20">
         <v>0.4</v>
@@ -2295,7 +2295,7 @@
         <v>2030</v>
       </c>
       <c r="F23" s="20">
-        <v>2030</v>
+        <v>2027</v>
       </c>
       <c r="G23" s="20">
         <v>1</v>
@@ -2430,7 +2430,7 @@
         <v>2030</v>
       </c>
       <c r="F26" s="20">
-        <v>2030</v>
+        <v>2027</v>
       </c>
       <c r="G26" s="20">
         <v>1</v>
@@ -2565,7 +2565,7 @@
         <v>2030</v>
       </c>
       <c r="F29" s="20">
-        <v>2030</v>
+        <v>2027</v>
       </c>
       <c r="G29" s="20">
         <v>1</v>

</xml_diff>

<commit_message>
Fixing EFF to be twh->PJ
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_NewTechs.xlsx
+++ b/SubRES_TMPL/SubRES_NewTechs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6376034-3F79-4321-8D26-5CAF0AC9069E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBB528E-7166-4011-877B-88D487515F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ELC" sheetId="4" r:id="rId1"/>
@@ -55,7 +55,7 @@
     Google otsing</t>
       </text>
     </comment>
-    <comment ref="I14" authorId="1" shapeId="0" xr:uid="{D5D738E1-1D01-4540-9F11-10D499C0D688}">
+    <comment ref="J14" authorId="1" shapeId="0" xr:uid="{D5D738E1-1D01-4540-9F11-10D499C0D688}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -63,7 +63,7 @@
     18 MUSD/MW</t>
       </text>
     </comment>
-    <comment ref="J14" authorId="2" shapeId="0" xr:uid="{A3E54751-892C-48B6-A7DF-516DEC7FED8F}">
+    <comment ref="K14" authorId="2" shapeId="0" xr:uid="{A3E54751-892C-48B6-A7DF-516DEC7FED8F}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -71,7 +71,7 @@
     Fermil oli antud 27 €/MWh kohta, mis sisaldas 6 €/Mwh kütusekulu </t>
       </text>
     </comment>
-    <comment ref="K14" authorId="3" shapeId="0" xr:uid="{7634B8F0-2D0A-458A-9170-2B40B7F18B83}">
+    <comment ref="L14" authorId="3" shapeId="0" xr:uid="{7634B8F0-2D0A-458A-9170-2B40B7F18B83}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="110">
   <si>
     <t>~FI_T</t>
   </si>
@@ -411,6 +411,9 @@
   </si>
   <si>
     <t>ELCWOF</t>
+  </si>
+  <si>
+    <t>TWh2PJ</t>
   </si>
 </sst>
 </file>
@@ -474,6 +477,8 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="186"/>
     </font>
     <font>
       <sz val="11"/>
@@ -573,7 +578,7 @@
       <charset val="186"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -610,6 +615,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -756,7 +767,7 @@
     <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -841,6 +852,17 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="30" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="8" borderId="0" xfId="15" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="15" applyFill="1"/>
   </cellXfs>
   <cellStyles count="56">
     <cellStyle name="20% - Accent5" xfId="1" builtinId="46"/>
@@ -1344,13 +1366,13 @@
   <threadedComment ref="G14" dT="2026-10-19T10:21:04.55" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{9A97F4CE-0467-4677-8B57-18CDF16525F8}">
     <text>Google otsing</text>
   </threadedComment>
-  <threadedComment ref="I14" dT="2026-10-19T10:23:13.18" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{D5D738E1-1D01-4540-9F11-10D499C0D688}">
+  <threadedComment ref="J14" dT="2026-10-19T10:23:13.18" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{D5D738E1-1D01-4540-9F11-10D499C0D688}">
     <text>18 MUSD/MW</text>
   </threadedComment>
-  <threadedComment ref="J14" dT="2026-10-19T10:37:46.35" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{A3E54751-892C-48B6-A7DF-516DEC7FED8F}">
+  <threadedComment ref="K14" dT="2026-10-19T10:37:46.35" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{A3E54751-892C-48B6-A7DF-516DEC7FED8F}">
     <text xml:space="preserve">Fermil oli antud 27 €/MWh kohta, mis sisaldas 6 €/Mwh kütusekulu </text>
   </threadedComment>
-  <threadedComment ref="K14" dT="2026-10-19T10:40:37.40" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{7634B8F0-2D0A-458A-9170-2B40B7F18B83}">
+  <threadedComment ref="L14" dT="2026-10-19T10:40:37.40" personId="{40B0B2C0-D4F7-40AE-B370-CC0D231C0275}" id="{7634B8F0-2D0A-458A-9170-2B40B7F18B83}">
     <text>google</text>
   </threadedComment>
 </ThreadedComments>
@@ -1359,7 +1381,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:Y31"/>
+  <dimension ref="A1:Z34"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" style="20" customWidth="1"/>
@@ -1367,31 +1389,32 @@
     <col min="3" max="3" width="18.28515625" style="20" customWidth="1"/>
     <col min="4" max="4" width="15.28515625" style="20" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" style="20" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="13.140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.7109375" style="20" customWidth="1"/>
-    <col min="9" max="9" width="10" style="20" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.28515625" style="20" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" style="20" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15" style="20" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" style="20" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="11.5703125" style="20" customWidth="1"/>
-    <col min="16" max="16" width="2" style="20" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.5703125" customWidth="1"/>
-    <col min="19" max="19" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="54.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.7109375" customWidth="1"/>
-    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.28515625" customWidth="1"/>
-    <col min="24" max="24" width="12.7109375" customWidth="1"/>
-    <col min="25" max="25" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" style="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" style="20" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" style="20" customWidth="1"/>
+    <col min="10" max="10" width="10" style="20" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.28515625" style="20" customWidth="1"/>
+    <col min="12" max="12" width="8.5703125" style="20" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15" style="20" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" style="20" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="11.5703125" style="20" customWidth="1"/>
+    <col min="17" max="17" width="2" style="20" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.5703125" customWidth="1"/>
+    <col min="20" max="20" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="54.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.7109375" customWidth="1"/>
+    <col min="23" max="23" width="10" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.28515625" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" customWidth="1"/>
+    <col min="26" max="26" width="7.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="23.25" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="Q2" s="27"/>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="R2" s="27"/>
       <c r="S2" s="27"/>
       <c r="T2" s="27"/>
@@ -1400,8 +1423,9 @@
       <c r="W2" s="27"/>
       <c r="X2" s="27"/>
       <c r="Y2" s="27"/>
-    </row>
-    <row r="3" spans="1:25" ht="15" x14ac:dyDescent="0.25">
+      <c r="Z2" s="27"/>
+    </row>
+    <row r="3" spans="1:26" ht="15" x14ac:dyDescent="0.25">
       <c r="B3" s="19" t="s">
         <v>42</v>
       </c>
@@ -1417,11 +1441,12 @@
       <c r="F3" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="G3" s="19"/>
+      <c r="I3" s="19" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="8" t="s">
         <v>47</v>
       </c>
@@ -1437,51 +1462,52 @@
       <c r="F4" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="G4" s="8"/>
+      <c r="I4" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="Q4" s="28" t="s">
+      <c r="R4" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="R4" s="28"/>
-      <c r="S4" s="29"/>
+      <c r="S4" s="28"/>
       <c r="T4" s="29"/>
       <c r="U4" s="29"/>
       <c r="V4" s="29"/>
       <c r="W4" s="29"/>
       <c r="X4" s="29"/>
       <c r="Y4" s="29"/>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="Q5" s="30" t="s">
+      <c r="Z4" s="29"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="R5" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="R5" s="31" t="s">
+      <c r="S5" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="S5" s="30" t="s">
+      <c r="T5" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="T5" s="30" t="s">
+      <c r="U5" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="U5" s="30" t="s">
+      <c r="V5" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="V5" s="30" t="s">
+      <c r="W5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="W5" s="30" t="s">
+      <c r="X5" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="X5" s="30" t="s">
+      <c r="Y5" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="Y5" s="30" t="s">
+      <c r="Z5" s="30" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="35.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" ht="35.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="24" t="s">
         <v>54</v>
       </c>
@@ -1494,36 +1520,36 @@
       <c r="E6" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="Q6" s="32" t="s">
+      <c r="H6" s="26"/>
+      <c r="R6" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="R6" s="32" t="s">
+      <c r="S6" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="S6" s="32" t="s">
+      <c r="T6" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="T6" s="32" t="s">
+      <c r="U6" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="U6" s="32" t="s">
+      <c r="V6" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="V6" s="32" t="s">
+      <c r="W6" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="W6" s="32" t="s">
+      <c r="X6" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="X6" s="32" t="s">
+      <c r="Y6" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="Y6" s="32" t="s">
+      <c r="Z6" s="32" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="23" t="s">
         <v>62</v>
       </c>
@@ -1536,42 +1562,49 @@
       <c r="E7" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="G7" s="25"/>
-      <c r="Q7" s="2"/>
-      <c r="S7" s="2"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="J7" s="20">
+        <v>3.6</v>
+      </c>
+      <c r="R7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
       <c r="X7" s="2"/>
       <c r="Y7" s="2"/>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="Q9" s="3"/>
+      <c r="Z7" s="2"/>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="R9" s="3"/>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="S9" s="3"/>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="E10" s="5" t="s">
         <v>0</v>
       </c>
       <c r="F10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="6"/>
+      <c r="G10" s="5"/>
+      <c r="I10" s="5"/>
       <c r="J10" s="6"/>
-      <c r="K10" s="4"/>
-      <c r="Q10" s="28" t="s">
+      <c r="K10" s="6"/>
+      <c r="L10" s="4"/>
+      <c r="R10" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="R10" s="28"/>
-      <c r="S10" s="29"/>
+      <c r="S10" s="28"/>
       <c r="T10" s="29"/>
       <c r="U10" s="29"/>
       <c r="V10" s="29"/>
       <c r="W10" s="29"/>
       <c r="X10" s="29"/>
       <c r="Y10" s="29"/>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="Z10" s="29"/>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B11" s="11" t="s">
         <v>1</v>
       </c>
@@ -1588,62 +1621,65 @@
         <v>15</v>
       </c>
       <c r="G11" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="H11" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="I11" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="J11" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="J11" s="14" t="s">
+      <c r="K11" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="K11" s="14" t="s">
+      <c r="L11" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="L11" s="13" t="s">
+      <c r="M11" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="M11" s="13" t="s">
+      <c r="N11" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N11" s="13" t="s">
+      <c r="O11" s="40" t="s">
         <v>67</v>
       </c>
-      <c r="O11" s="13" t="s">
+      <c r="P11" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="P11" s="21"/>
-      <c r="Q11" s="30" t="s">
+      <c r="Q11" s="21"/>
+      <c r="R11" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="R11" s="31" t="s">
+      <c r="S11" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="S11" s="30" t="s">
+      <c r="T11" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="T11" s="30" t="s">
+      <c r="U11" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="U11" s="30" t="s">
+      <c r="V11" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="V11" s="30" t="s">
+      <c r="W11" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="W11" s="30" t="s">
+      <c r="X11" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="X11" s="30" t="s">
+      <c r="Y11" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="Y11" s="30" t="s">
+      <c r="Z11" s="30" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:26" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="10" t="s">
         <v>68</v>
       </c>
@@ -1657,62 +1693,63 @@
       <c r="F12" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="G12" s="15"/>
+      <c r="H12" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="H12" s="16" t="s">
+      <c r="I12" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="J12" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="J12" s="15" t="s">
+      <c r="K12" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="K12" s="15" t="s">
+      <c r="L12" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="L12" s="15" t="s">
+      <c r="M12" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="M12" s="15" t="s">
+      <c r="N12" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="N12" s="15" t="s">
+      <c r="O12" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="O12" s="39" t="s">
+      <c r="P12" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="Q12" s="33" t="s">
+      <c r="R12" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="R12" s="33" t="s">
+      <c r="S12" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="S12" s="33" t="s">
+      <c r="T12" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="T12" s="33" t="s">
+      <c r="U12" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="U12" s="33" t="s">
+      <c r="V12" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="V12" s="33" t="s">
+      <c r="W12" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="W12" s="33" t="s">
+      <c r="X12" s="33" t="s">
         <v>73</v>
       </c>
-      <c r="X12" s="33" t="s">
+      <c r="Y12" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="Y12" s="33" t="s">
+      <c r="Z12" s="33" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>75</v>
       </c>
@@ -1721,28 +1758,28 @@
       <c r="E13" s="9"/>
       <c r="F13" s="17"/>
       <c r="G13" s="17"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="17" t="s">
-        <v>76</v>
-      </c>
+      <c r="H13" s="17"/>
+      <c r="I13" s="18"/>
       <c r="J13" s="17" t="s">
         <v>76</v>
       </c>
       <c r="K13" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="L13" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="L13" s="17" t="s">
+      <c r="M13" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="M13" s="17" t="s">
+      <c r="N13" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="N13" s="17"/>
-      <c r="O13" s="17"/>
-      <c r="Q13" s="32" t="s">
+      <c r="O13" s="42"/>
+      <c r="P13" s="17"/>
+      <c r="R13" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="R13" s="32"/>
       <c r="S13" s="32"/>
       <c r="T13" s="32"/>
       <c r="U13" s="32"/>
@@ -1750,10 +1787,11 @@
       <c r="W13" s="32"/>
       <c r="X13" s="32"/>
       <c r="Y13" s="32"/>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="Z13" s="32"/>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B14" s="36" t="str">
-        <f>$S$14</f>
+        <f>$T$14</f>
         <v>ELC_FERMI_SMR</v>
       </c>
       <c r="C14" s="20" t="s">
@@ -1772,55 +1810,59 @@
         <v>0.3</v>
       </c>
       <c r="H14" s="20">
+        <f>G14*$J$7</f>
+        <v>1.08</v>
+      </c>
+      <c r="I14" s="20">
         <v>0.92</v>
       </c>
-      <c r="I14" s="20">
+      <c r="J14" s="20">
         <v>15000</v>
       </c>
-      <c r="J14" s="22">
-        <f>21*H14*8760*1000/1000000</f>
+      <c r="K14" s="22">
+        <f>21*I14*8760*1000/1000000</f>
         <v>169.2432</v>
       </c>
-      <c r="K14" s="22">
+      <c r="L14" s="22">
         <v>3.15</v>
       </c>
-      <c r="L14" s="20">
+      <c r="M14" s="20">
         <v>60</v>
       </c>
-      <c r="M14" s="20">
+      <c r="N14" s="20">
         <v>8.76</v>
       </c>
-      <c r="N14" s="22">
+      <c r="O14" s="43">
         <v>1</v>
       </c>
-      <c r="O14" s="22"/>
-      <c r="Q14" s="35" t="s">
+      <c r="P14" s="22"/>
+      <c r="R14" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="R14" s="34"/>
-      <c r="S14" s="36" t="s">
+      <c r="S14" s="34"/>
+      <c r="T14" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="T14" s="34" t="s">
+      <c r="U14" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="U14" s="34" t="s">
+      <c r="V14" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="V14" s="34" t="s">
+      <c r="W14" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="W14" t="s">
+      <c r="X14" t="s">
         <v>90</v>
       </c>
-      <c r="X14" s="34"/>
-      <c r="Y14" s="34" t="s">
+      <c r="Y14" s="34"/>
+      <c r="Z14" s="34" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B15" s="36" t="str">
-        <f>$S$14</f>
+        <f>$T$14</f>
         <v>ELC_FERMI_SMR</v>
       </c>
       <c r="C15" s="20" t="s">
@@ -1836,54 +1878,58 @@
         <v>0.3</v>
       </c>
       <c r="H15" s="20">
+        <f t="shared" ref="H15:H31" si="0">G15*$J$7</f>
+        <v>1.08</v>
+      </c>
+      <c r="I15" s="20">
         <v>0.92</v>
       </c>
-      <c r="I15" s="20">
+      <c r="J15" s="20">
         <v>15000</v>
       </c>
-      <c r="J15" s="22">
-        <f t="shared" ref="J15:J16" si="0">169243*1000/1000000</f>
+      <c r="K15" s="22">
+        <f t="shared" ref="K15:K16" si="1">169243*1000/1000000</f>
         <v>169.24299999999999</v>
       </c>
-      <c r="K15" s="22">
+      <c r="L15" s="22">
         <v>3.15</v>
       </c>
-      <c r="L15" s="20">
+      <c r="M15" s="20">
         <v>60</v>
       </c>
-      <c r="M15" s="20">
+      <c r="N15" s="20">
         <v>8.76</v>
       </c>
-      <c r="N15" s="22">
+      <c r="O15" s="43">
         <v>1</v>
       </c>
-      <c r="O15" s="22"/>
-      <c r="Q15" s="38" t="s">
+      <c r="P15" s="22"/>
+      <c r="R15" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="S15" s="20" t="s">
+      <c r="T15" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="T15" t="s">
+      <c r="U15" t="s">
         <v>94</v>
       </c>
-      <c r="U15" s="34" t="s">
+      <c r="V15" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="V15" s="34" t="s">
+      <c r="W15" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="W15" t="s">
+      <c r="X15" t="s">
         <v>90</v>
       </c>
-      <c r="X15" s="34"/>
-      <c r="Y15" s="34" t="s">
+      <c r="Y15" s="34"/>
+      <c r="Z15" s="34" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B16" s="36" t="str">
-        <f>$S$14</f>
+        <f>$T$14</f>
         <v>ELC_FERMI_SMR</v>
       </c>
       <c r="C16" s="20" t="s">
@@ -1899,54 +1945,58 @@
         <v>0.3</v>
       </c>
       <c r="H16" s="20">
+        <f t="shared" si="0"/>
+        <v>1.08</v>
+      </c>
+      <c r="I16" s="20">
         <v>0.92</v>
       </c>
-      <c r="I16" s="20">
+      <c r="J16" s="20">
         <v>15000</v>
       </c>
-      <c r="J16" s="22">
-        <f t="shared" si="0"/>
+      <c r="K16" s="22">
+        <f t="shared" si="1"/>
         <v>169.24299999999999</v>
       </c>
-      <c r="K16" s="22">
+      <c r="L16" s="22">
         <v>3.15</v>
       </c>
-      <c r="L16" s="20">
+      <c r="M16" s="20">
         <v>60</v>
       </c>
-      <c r="M16" s="20">
+      <c r="N16" s="20">
         <v>8.76</v>
       </c>
-      <c r="N16" s="22">
+      <c r="O16" s="43">
         <v>1</v>
       </c>
-      <c r="O16" s="22"/>
-      <c r="Q16" s="38" t="s">
+      <c r="P16" s="22"/>
+      <c r="R16" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="S16" s="38" t="s">
+      <c r="T16" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="T16" s="38" t="s">
+      <c r="U16" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="U16" s="34" t="s">
+      <c r="V16" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="V16" s="34" t="s">
+      <c r="W16" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="W16" t="s">
+      <c r="X16" t="s">
         <v>90</v>
       </c>
-      <c r="X16" s="34"/>
-      <c r="Y16" s="34" t="s">
+      <c r="Y16" s="34"/>
+      <c r="Z16" s="34" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B17" s="20" t="str">
-        <f>$S$15</f>
+        <f>$T$15</f>
         <v>ELC_CCGT_PP</v>
       </c>
       <c r="C17" s="20" t="s">
@@ -1965,57 +2015,61 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="H17" s="20">
+        <f t="shared" si="0"/>
+        <v>2.0160000000000005</v>
+      </c>
+      <c r="I17" s="20">
         <v>0.97</v>
       </c>
-      <c r="I17" s="20">
+      <c r="J17" s="20">
         <f>1.2*1000</f>
         <v>1200</v>
       </c>
-      <c r="J17" s="22">
+      <c r="K17" s="22">
         <f>39143*1000/1000000</f>
         <v>39.143000000000001</v>
       </c>
-      <c r="K17" s="20">
+      <c r="L17" s="20">
         <v>5.9</v>
       </c>
-      <c r="L17" s="20">
+      <c r="M17" s="20">
         <v>25</v>
       </c>
-      <c r="M17" s="20">
+      <c r="N17" s="20">
         <v>8.76</v>
       </c>
-      <c r="N17" s="22">
+      <c r="O17" s="43">
         <v>1</v>
       </c>
-      <c r="O17" s="22">
+      <c r="P17" s="22">
         <v>2.5</v>
       </c>
-      <c r="Q17" s="38" t="s">
+      <c r="R17" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="S17" s="38" t="s">
+      <c r="T17" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="T17" s="38" t="s">
+      <c r="U17" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="U17" s="34" t="s">
+      <c r="V17" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="V17" s="34" t="s">
+      <c r="W17" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="W17" t="s">
+      <c r="X17" t="s">
         <v>90</v>
       </c>
-      <c r="X17" s="34"/>
-      <c r="Y17" s="34" t="s">
+      <c r="Y17" s="34"/>
+      <c r="Z17" s="34" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="18" spans="2:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="20" t="str">
-        <f>$S$15</f>
+        <f>$T$15</f>
         <v>ELC_CCGT_PP</v>
       </c>
       <c r="C18" s="20" t="s">
@@ -2031,57 +2085,61 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="H18" s="20">
+        <f t="shared" si="0"/>
+        <v>2.0160000000000005</v>
+      </c>
+      <c r="I18" s="20">
         <v>0.97</v>
       </c>
-      <c r="I18" s="20">
+      <c r="J18" s="20">
         <f>1.2*1000</f>
         <v>1200</v>
       </c>
-      <c r="J18" s="22">
-        <f t="shared" ref="J18:J19" si="1">39143*1000/1000000</f>
+      <c r="K18" s="22">
+        <f t="shared" ref="K18:K19" si="2">39143*1000/1000000</f>
         <v>39.143000000000001</v>
       </c>
-      <c r="K18" s="20">
+      <c r="L18" s="20">
         <v>5.9</v>
       </c>
-      <c r="L18" s="20">
+      <c r="M18" s="20">
         <v>25</v>
       </c>
-      <c r="M18" s="20">
+      <c r="N18" s="20">
         <v>8.76</v>
       </c>
-      <c r="N18" s="22">
+      <c r="O18" s="43">
         <v>1</v>
       </c>
-      <c r="O18" s="22">
+      <c r="P18" s="22">
         <v>2.5</v>
       </c>
-      <c r="Q18" s="38" t="s">
+      <c r="R18" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="S18" s="20" t="s">
+      <c r="T18" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="T18" s="20" t="s">
+      <c r="U18" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="U18" s="34" t="s">
+      <c r="V18" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="V18" s="34" t="s">
+      <c r="W18" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="W18" t="s">
+      <c r="X18" t="s">
         <v>90</v>
       </c>
-      <c r="X18" s="34"/>
-      <c r="Y18" s="34" t="s">
+      <c r="Y18" s="34"/>
+      <c r="Z18" s="34" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="2:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="20" t="str">
-        <f>$S$15</f>
+        <f>$T$15</f>
         <v>ELC_CCGT_PP</v>
       </c>
       <c r="C19" s="20" t="s">
@@ -2097,57 +2155,61 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="H19" s="20">
+        <f t="shared" si="0"/>
+        <v>2.0160000000000005</v>
+      </c>
+      <c r="I19" s="20">
         <v>0.97</v>
       </c>
-      <c r="I19" s="20">
+      <c r="J19" s="20">
         <f>1.2*1000</f>
         <v>1200</v>
       </c>
-      <c r="J19" s="22">
-        <f t="shared" si="1"/>
+      <c r="K19" s="22">
+        <f t="shared" si="2"/>
         <v>39.143000000000001</v>
       </c>
-      <c r="K19" s="20">
+      <c r="L19" s="20">
         <v>5.9</v>
       </c>
-      <c r="L19" s="20">
+      <c r="M19" s="20">
         <v>25</v>
       </c>
-      <c r="M19" s="20">
+      <c r="N19" s="20">
         <v>8.76</v>
       </c>
-      <c r="N19" s="22">
+      <c r="O19" s="43">
         <v>1</v>
       </c>
-      <c r="O19" s="22">
+      <c r="P19" s="22">
         <v>2.5</v>
       </c>
-      <c r="Q19" s="38" t="s">
+      <c r="R19" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="S19" s="38" t="s">
+      <c r="T19" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="T19" s="38" t="s">
+      <c r="U19" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="U19" s="34" t="s">
+      <c r="V19" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="V19" s="34" t="s">
+      <c r="W19" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="W19" t="s">
+      <c r="X19" t="s">
         <v>90</v>
       </c>
-      <c r="X19" s="34"/>
-      <c r="Y19" s="34" t="s">
+      <c r="Y19" s="34"/>
+      <c r="Z19" s="34" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B20" s="20" t="str">
-        <f>$S$16</f>
+        <f>$T$16</f>
         <v>ELC_OCGT_PP</v>
       </c>
       <c r="C20" s="20" t="s">
@@ -2166,35 +2228,39 @@
         <v>0.4</v>
       </c>
       <c r="H20" s="20">
+        <f t="shared" si="0"/>
+        <v>1.4400000000000002</v>
+      </c>
+      <c r="I20" s="20">
         <v>0.99</v>
       </c>
-      <c r="I20" s="20">
+      <c r="J20" s="20">
         <f>0.6*1000</f>
         <v>600</v>
       </c>
-      <c r="J20" s="22">
+      <c r="K20" s="22">
         <f>10778*1000/1000000</f>
         <v>10.778</v>
       </c>
-      <c r="K20" s="37">
+      <c r="L20" s="37">
         <v>6</v>
       </c>
-      <c r="L20" s="20">
+      <c r="M20" s="20">
         <v>25</v>
       </c>
-      <c r="M20" s="20">
+      <c r="N20" s="20">
         <v>8.76</v>
       </c>
-      <c r="N20" s="22">
+      <c r="O20" s="43">
         <v>1</v>
       </c>
-      <c r="O20" s="20">
+      <c r="P20" s="20">
         <v>0.2</v>
       </c>
     </row>
-    <row r="21" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B21" s="20" t="str">
-        <f t="shared" ref="B21:B22" si="2">$S$16</f>
+        <f t="shared" ref="B21:B22" si="3">$T$16</f>
         <v>ELC_OCGT_PP</v>
       </c>
       <c r="C21" s="20" t="s">
@@ -2210,35 +2276,39 @@
         <v>0.4</v>
       </c>
       <c r="H21" s="20">
+        <f t="shared" si="0"/>
+        <v>1.4400000000000002</v>
+      </c>
+      <c r="I21" s="20">
         <v>0.99</v>
       </c>
-      <c r="I21" s="20">
-        <f t="shared" ref="I21:I22" si="3">0.6*1000</f>
+      <c r="J21" s="20">
+        <f t="shared" ref="J21:J22" si="4">0.6*1000</f>
         <v>600</v>
       </c>
-      <c r="J21" s="22">
-        <f t="shared" ref="J21:J22" si="4">10778*1000/1000000</f>
+      <c r="K21" s="22">
+        <f t="shared" ref="K21:K22" si="5">10778*1000/1000000</f>
         <v>10.778</v>
       </c>
-      <c r="K21" s="37">
+      <c r="L21" s="37">
         <v>6</v>
       </c>
-      <c r="L21" s="20">
+      <c r="M21" s="20">
         <v>25</v>
       </c>
-      <c r="M21" s="20">
+      <c r="N21" s="20">
         <v>8.76</v>
       </c>
-      <c r="N21" s="22">
+      <c r="O21" s="43">
         <v>1</v>
       </c>
-      <c r="O21" s="20">
+      <c r="P21" s="20">
         <v>0.2</v>
       </c>
     </row>
-    <row r="22" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>ELC_OCGT_PP</v>
       </c>
       <c r="C22" s="20" t="s">
@@ -2254,35 +2324,39 @@
         <v>0.4</v>
       </c>
       <c r="H22" s="20">
+        <f t="shared" si="0"/>
+        <v>1.4400000000000002</v>
+      </c>
+      <c r="I22" s="20">
         <v>0.99</v>
       </c>
-      <c r="I22" s="20">
-        <f t="shared" si="3"/>
+      <c r="J22" s="20">
+        <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="J22" s="22">
-        <f t="shared" si="4"/>
+      <c r="K22" s="22">
+        <f t="shared" si="5"/>
         <v>10.778</v>
       </c>
-      <c r="K22" s="37">
+      <c r="L22" s="37">
         <v>6</v>
       </c>
-      <c r="L22" s="20">
+      <c r="M22" s="20">
         <v>25</v>
       </c>
-      <c r="M22" s="20">
+      <c r="N22" s="20">
         <v>8.76</v>
       </c>
-      <c r="N22" s="22">
+      <c r="O22" s="43">
         <v>1</v>
       </c>
-      <c r="O22" s="20">
+      <c r="P22" s="20">
         <v>0.2</v>
       </c>
     </row>
-    <row r="23" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B23" s="20" t="str">
-        <f>$S$17</f>
+        <f>$T$17</f>
         <v>ELC_PV_UTIL</v>
       </c>
       <c r="C23" s="20" t="s">
@@ -2301,35 +2375,39 @@
         <v>1</v>
       </c>
       <c r="H23" s="20">
+        <f t="shared" si="0"/>
+        <v>3.6</v>
+      </c>
+      <c r="I23" s="20">
         <v>0.3</v>
       </c>
-      <c r="I23" s="20">
+      <c r="J23" s="20">
         <f>0.7*1000</f>
         <v>700</v>
       </c>
-      <c r="J23" s="22">
+      <c r="K23" s="22">
         <f>12601*1000/1000000</f>
         <v>12.601000000000001</v>
       </c>
-      <c r="K23" s="20">
+      <c r="L23" s="20">
         <v>0</v>
       </c>
-      <c r="L23" s="20">
+      <c r="M23" s="20">
         <v>40</v>
       </c>
-      <c r="M23" s="20">
+      <c r="N23" s="20">
         <v>8.76</v>
       </c>
-      <c r="N23" s="22">
+      <c r="O23" s="43">
         <v>0.15</v>
       </c>
-      <c r="O23" s="20">
+      <c r="P23" s="20">
         <v>0.5</v>
       </c>
     </row>
-    <row r="24" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B24" s="20" t="str">
-        <f t="shared" ref="B24:B25" si="5">$S$17</f>
+        <f t="shared" ref="B24:B25" si="6">$T$17</f>
         <v>ELC_PV_UTIL</v>
       </c>
       <c r="C24" s="20" t="s">
@@ -2345,35 +2423,39 @@
         <v>1</v>
       </c>
       <c r="H24" s="20">
+        <f t="shared" si="0"/>
+        <v>3.6</v>
+      </c>
+      <c r="I24" s="20">
         <v>0.3</v>
       </c>
-      <c r="I24" s="20">
-        <f t="shared" ref="I24:I25" si="6">0.7*1000</f>
+      <c r="J24" s="20">
+        <f t="shared" ref="J24:J25" si="7">0.7*1000</f>
         <v>700</v>
       </c>
-      <c r="J24" s="22">
-        <f t="shared" ref="J24:J25" si="7">12601*1000/1000000</f>
+      <c r="K24" s="22">
+        <f t="shared" ref="K24:K25" si="8">12601*1000/1000000</f>
         <v>12.601000000000001</v>
       </c>
-      <c r="K24" s="20">
+      <c r="L24" s="20">
         <v>0</v>
       </c>
-      <c r="L24" s="20">
+      <c r="M24" s="20">
         <v>40</v>
       </c>
-      <c r="M24" s="20">
+      <c r="N24" s="20">
         <v>8.76</v>
       </c>
-      <c r="N24" s="22">
+      <c r="O24" s="43">
         <v>0.15</v>
       </c>
-      <c r="O24" s="20">
+      <c r="P24" s="20">
         <v>0.5</v>
       </c>
     </row>
-    <row r="25" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B25" s="20" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>ELC_PV_UTIL</v>
       </c>
       <c r="C25" s="20" t="s">
@@ -2389,35 +2471,39 @@
         <v>1</v>
       </c>
       <c r="H25" s="20">
+        <f t="shared" si="0"/>
+        <v>3.6</v>
+      </c>
+      <c r="I25" s="20">
         <v>0.3</v>
       </c>
-      <c r="I25" s="20">
-        <f t="shared" si="6"/>
+      <c r="J25" s="20">
+        <f t="shared" si="7"/>
         <v>700</v>
       </c>
-      <c r="J25" s="22">
-        <f t="shared" si="7"/>
+      <c r="K25" s="22">
+        <f t="shared" si="8"/>
         <v>12.601000000000001</v>
       </c>
-      <c r="K25" s="20">
+      <c r="L25" s="20">
         <v>0</v>
       </c>
-      <c r="L25" s="20">
+      <c r="M25" s="20">
         <v>40</v>
       </c>
-      <c r="M25" s="20">
+      <c r="N25" s="20">
         <v>8.76</v>
       </c>
-      <c r="N25" s="22">
+      <c r="O25" s="43">
         <v>0.15</v>
       </c>
-      <c r="O25" s="20">
+      <c r="P25" s="20">
         <v>0.5</v>
       </c>
     </row>
-    <row r="26" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="str">
-        <f>$S$18</f>
+        <f>$T$18</f>
         <v>ELC_WON_PP</v>
       </c>
       <c r="C26" s="20" t="s">
@@ -2436,35 +2522,39 @@
         <v>1</v>
       </c>
       <c r="H26" s="20">
+        <f t="shared" si="0"/>
+        <v>3.6</v>
+      </c>
+      <c r="I26" s="20">
         <v>0.3</v>
       </c>
-      <c r="I26" s="20">
+      <c r="J26" s="20">
         <f>1.5*1000</f>
         <v>1500</v>
       </c>
-      <c r="J26" s="22">
+      <c r="K26" s="22">
         <f>21843*1000/1000000</f>
         <v>21.843</v>
       </c>
-      <c r="K26" s="20">
+      <c r="L26" s="20">
         <v>2.6</v>
       </c>
-      <c r="L26" s="20">
+      <c r="M26" s="20">
         <v>27</v>
       </c>
-      <c r="M26" s="20">
+      <c r="N26" s="20">
         <v>8.76</v>
       </c>
-      <c r="N26" s="22">
+      <c r="O26" s="43">
         <v>0.4</v>
       </c>
-      <c r="O26" s="20">
+      <c r="P26" s="20">
         <v>1.5</v>
       </c>
     </row>
-    <row r="27" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B27" s="20" t="str">
-        <f t="shared" ref="B27:B28" si="8">$S$18</f>
+        <f t="shared" ref="B27:B28" si="9">$T$18</f>
         <v>ELC_WON_PP</v>
       </c>
       <c r="C27" s="20" t="s">
@@ -2480,35 +2570,39 @@
         <v>1</v>
       </c>
       <c r="H27" s="20">
+        <f t="shared" si="0"/>
+        <v>3.6</v>
+      </c>
+      <c r="I27" s="20">
         <v>0.3</v>
       </c>
-      <c r="I27" s="20">
-        <f t="shared" ref="I27:I28" si="9">1.5*1000</f>
+      <c r="J27" s="20">
+        <f t="shared" ref="J27:J28" si="10">1.5*1000</f>
         <v>1500</v>
       </c>
-      <c r="J27" s="22">
-        <f t="shared" ref="J27:J28" si="10">21843*1000/1000000</f>
+      <c r="K27" s="22">
+        <f t="shared" ref="K27:K28" si="11">21843*1000/1000000</f>
         <v>21.843</v>
       </c>
-      <c r="K27" s="20">
+      <c r="L27" s="20">
         <v>2.6</v>
       </c>
-      <c r="L27" s="20">
+      <c r="M27" s="20">
         <v>27</v>
       </c>
-      <c r="M27" s="20">
+      <c r="N27" s="20">
         <v>8.76</v>
       </c>
-      <c r="N27" s="22">
+      <c r="O27" s="43">
         <v>0.4</v>
       </c>
-      <c r="O27" s="20">
+      <c r="P27" s="20">
         <v>1.5</v>
       </c>
     </row>
-    <row r="28" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>ELC_WON_PP</v>
       </c>
       <c r="C28" s="20" t="s">
@@ -2524,35 +2618,39 @@
         <v>1</v>
       </c>
       <c r="H28" s="20">
+        <f t="shared" si="0"/>
+        <v>3.6</v>
+      </c>
+      <c r="I28" s="20">
         <v>0.3</v>
       </c>
-      <c r="I28" s="20">
-        <f t="shared" si="9"/>
+      <c r="J28" s="20">
+        <f t="shared" si="10"/>
         <v>1500</v>
       </c>
-      <c r="J28" s="22">
-        <f t="shared" si="10"/>
+      <c r="K28" s="22">
+        <f t="shared" si="11"/>
         <v>21.843</v>
       </c>
-      <c r="K28" s="20">
+      <c r="L28" s="20">
         <v>2.6</v>
       </c>
-      <c r="L28" s="20">
+      <c r="M28" s="20">
         <v>27</v>
       </c>
-      <c r="M28" s="20">
+      <c r="N28" s="20">
         <v>8.76</v>
       </c>
-      <c r="N28" s="22">
+      <c r="O28" s="43">
         <v>0.4</v>
       </c>
-      <c r="O28" s="20">
+      <c r="P28" s="20">
         <v>1.5</v>
       </c>
     </row>
-    <row r="29" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B29" s="20" t="str">
-        <f>$S$19</f>
+        <f>$T$19</f>
         <v>ELC_WOF_PP</v>
       </c>
       <c r="C29" s="20" t="s">
@@ -2571,35 +2669,39 @@
         <v>1</v>
       </c>
       <c r="H29" s="20">
+        <f t="shared" si="0"/>
+        <v>3.6</v>
+      </c>
+      <c r="I29" s="20">
         <v>0.3</v>
       </c>
-      <c r="I29" s="20">
+      <c r="J29" s="20">
         <f>3.5*1000</f>
         <v>3500</v>
       </c>
-      <c r="J29" s="22">
+      <c r="K29" s="22">
         <f>55278*1000/1000000</f>
         <v>55.277999999999999</v>
       </c>
-      <c r="K29" s="20">
+      <c r="L29" s="20">
         <v>5.5</v>
       </c>
-      <c r="L29" s="20">
+      <c r="M29" s="20">
         <v>30</v>
       </c>
-      <c r="M29" s="20">
+      <c r="N29" s="20">
         <v>8.76</v>
       </c>
-      <c r="N29" s="22">
+      <c r="O29" s="43">
         <v>0.4</v>
       </c>
-      <c r="O29" s="20">
+      <c r="P29" s="20">
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="str">
-        <f>$S$19</f>
+        <f>$T$19</f>
         <v>ELC_WOF_PP</v>
       </c>
       <c r="C30" s="20" t="s">
@@ -2615,35 +2717,39 @@
         <v>1</v>
       </c>
       <c r="H30" s="20">
+        <f t="shared" si="0"/>
+        <v>3.6</v>
+      </c>
+      <c r="I30" s="20">
         <v>0.3</v>
       </c>
-      <c r="I30" s="20">
-        <f t="shared" ref="I30:I31" si="11">3.5*1000</f>
+      <c r="J30" s="20">
+        <f t="shared" ref="J30:J31" si="12">3.5*1000</f>
         <v>3500</v>
       </c>
-      <c r="J30" s="22">
-        <f t="shared" ref="J30:J31" si="12">55278*1000/1000000</f>
+      <c r="K30" s="22">
+        <f t="shared" ref="K30:K31" si="13">55278*1000/1000000</f>
         <v>55.277999999999999</v>
       </c>
-      <c r="K30" s="20">
+      <c r="L30" s="20">
         <v>5.5</v>
       </c>
-      <c r="L30" s="20">
+      <c r="M30" s="20">
         <v>30</v>
       </c>
-      <c r="M30" s="20">
+      <c r="N30" s="20">
         <v>8.76</v>
       </c>
-      <c r="N30" s="22">
+      <c r="O30" s="43">
         <v>0.4</v>
       </c>
-      <c r="O30" s="20">
+      <c r="P30" s="20">
         <v>3.5</v>
       </c>
     </row>
-    <row r="31" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B31" s="20" t="str">
-        <f>$S$19</f>
+        <f>$T$19</f>
         <v>ELC_WOF_PP</v>
       </c>
       <c r="C31" s="20" t="s">
@@ -2659,31 +2765,44 @@
         <v>1</v>
       </c>
       <c r="H31" s="20">
+        <f t="shared" si="0"/>
+        <v>3.6</v>
+      </c>
+      <c r="I31" s="20">
         <v>0.3</v>
       </c>
-      <c r="I31" s="20">
-        <f t="shared" si="11"/>
+      <c r="J31" s="20">
+        <f t="shared" si="12"/>
         <v>3500</v>
       </c>
-      <c r="J31" s="22">
-        <f t="shared" si="12"/>
+      <c r="K31" s="22">
+        <f t="shared" si="13"/>
         <v>55.277999999999999</v>
       </c>
-      <c r="K31" s="20">
+      <c r="L31" s="20">
         <v>5.5</v>
       </c>
-      <c r="L31" s="20">
+      <c r="M31" s="20">
         <v>30</v>
       </c>
-      <c r="M31" s="20">
+      <c r="N31" s="20">
         <v>8.76</v>
       </c>
-      <c r="N31" s="22">
+      <c r="O31" s="43">
         <v>0.4</v>
       </c>
-      <c r="O31" s="20">
+      <c r="P31" s="20">
         <v>3.5</v>
       </c>
+    </row>
+    <row r="32" spans="2:26" x14ac:dyDescent="0.2">
+      <c r="O32" s="44"/>
+    </row>
+    <row r="33" spans="15:15" x14ac:dyDescent="0.2">
+      <c r="O33" s="44"/>
+    </row>
+    <row r="34" spans="15:15" x14ac:dyDescent="0.2">
+      <c r="O34" s="44"/>
     </row>
   </sheetData>
   <phoneticPr fontId="0" type="noConversion"/>

</xml_diff>